<commit_message>
Fix:Fixed the email error
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -537,9 +537,78 @@
         <v>No</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>shravan</v>
+      </c>
+      <c r="B7" t="str">
+        <v>175</v>
+      </c>
+      <c r="C7" t="str">
+        <v>sniperkraken007@gmail.com</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Veg</v>
+      </c>
+      <c r="E7">
+        <v>321</v>
+      </c>
+      <c r="F7" t="str">
+        <v>160fc85e-1772-4f83-a920-0df6c85d5793</v>
+      </c>
+      <c r="G7" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Shravan R</v>
+      </c>
+      <c r="B8" t="str">
+        <v>175</v>
+      </c>
+      <c r="C8" t="str">
+        <v>sniperkraken007@gmail.com</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Veg</v>
+      </c>
+      <c r="E8">
+        <v>693</v>
+      </c>
+      <c r="F8" t="str">
+        <v>856d90b7-4506-4351-a017-2a16beaa2279</v>
+      </c>
+      <c r="G8" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Shravan R</v>
+      </c>
+      <c r="B9" t="str">
+        <v>175</v>
+      </c>
+      <c r="C9" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Non-Veg</v>
+      </c>
+      <c r="E9">
+        <v>746</v>
+      </c>
+      <c r="F9" t="str">
+        <v>eb258263-2334-4d6b-8b18-5bda969e00cd</v>
+      </c>
+      <c r="G9" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Feat: Delete column in the admin dashboard
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,10 +436,10 @@
         <v>Veg</v>
       </c>
       <c r="E2">
-        <v>484</v>
+        <v>620</v>
       </c>
       <c r="F2" t="str">
-        <v>cb19e59c-f5f9-434f-9f91-fc0f94e19a1a</v>
+        <v>db484a6e-f78d-4fed-abd4-82d76873e244</v>
       </c>
       <c r="G2" t="str">
         <v>No</v>
@@ -447,7 +447,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Shravan R</v>
+        <v>shravan</v>
       </c>
       <c r="B3" t="str">
         <v>175</v>
@@ -459,10 +459,10 @@
         <v>Veg</v>
       </c>
       <c r="E3">
-        <v>599</v>
+        <v>816</v>
       </c>
       <c r="F3" t="str">
-        <v>d1e991d4-d219-458d-87d8-9b0af4fd9e65</v>
+        <v>0d1498e1-aef8-4097-912a-d99cab0f3b85</v>
       </c>
       <c r="G3" t="str">
         <v>No</v>
@@ -476,16 +476,16 @@
         <v>175</v>
       </c>
       <c r="C4" t="str">
-        <v>sniperkraken007@gmail.com</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D4" t="str">
         <v>Veg</v>
       </c>
       <c r="E4">
-        <v>620</v>
+        <v>507</v>
       </c>
       <c r="F4" t="str">
-        <v>db484a6e-f78d-4fed-abd4-82d76873e244</v>
+        <v>0649a2f2-a85c-48e4-a00d-9c899f1139df</v>
       </c>
       <c r="G4" t="str">
         <v>No</v>
@@ -505,10 +505,10 @@
         <v>Veg</v>
       </c>
       <c r="E5">
-        <v>816</v>
+        <v>321</v>
       </c>
       <c r="F5" t="str">
-        <v>0d1498e1-aef8-4097-912a-d99cab0f3b85</v>
+        <v>160fc85e-1772-4f83-a920-0df6c85d5793</v>
       </c>
       <c r="G5" t="str">
         <v>No</v>
@@ -522,16 +522,16 @@
         <v>175</v>
       </c>
       <c r="C6" t="str">
-        <v>shravanramakunja@gmail.com</v>
+        <v>sniperkraken007@gmail.com</v>
       </c>
       <c r="D6" t="str">
         <v>Veg</v>
       </c>
       <c r="E6">
-        <v>507</v>
+        <v>693</v>
       </c>
       <c r="F6" t="str">
-        <v>0649a2f2-a85c-48e4-a00d-9c899f1139df</v>
+        <v>856d90b7-4506-4351-a017-2a16beaa2279</v>
       </c>
       <c r="G6" t="str">
         <v>No</v>
@@ -539,22 +539,22 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>shravan</v>
+        <v>Shravan R</v>
       </c>
       <c r="B7" t="str">
         <v>175</v>
       </c>
       <c r="C7" t="str">
-        <v>sniperkraken007@gmail.com</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D7" t="str">
-        <v>Veg</v>
+        <v>Non-Veg</v>
       </c>
       <c r="E7">
-        <v>321</v>
+        <v>746</v>
       </c>
       <c r="F7" t="str">
-        <v>160fc85e-1772-4f83-a920-0df6c85d5793</v>
+        <v>eb258263-2334-4d6b-8b18-5bda969e00cd</v>
       </c>
       <c r="G7" t="str">
         <v>No</v>
@@ -562,10 +562,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Shravan R</v>
+        <v>Sniper Kraken</v>
       </c>
       <c r="B8" t="str">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C8" t="str">
         <v>sniperkraken007@gmail.com</v>
@@ -574,64 +574,18 @@
         <v>Veg</v>
       </c>
       <c r="E8">
-        <v>693</v>
+        <v>967</v>
       </c>
       <c r="F8" t="str">
-        <v>856d90b7-4506-4351-a017-2a16beaa2279</v>
+        <v>78a002bd-67a3-40bd-a81d-2d5b77f1ea67</v>
       </c>
       <c r="G8" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Shravan R</v>
-      </c>
-      <c r="B9" t="str">
-        <v>175</v>
-      </c>
-      <c r="C9" t="str">
-        <v>shravanramakunja@gmail.com</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Non-Veg</v>
-      </c>
-      <c r="E9">
-        <v>746</v>
-      </c>
-      <c r="F9" t="str">
-        <v>eb258263-2334-4d6b-8b18-5bda969e00cd</v>
-      </c>
-      <c r="G9" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Sniper Kraken</v>
-      </c>
-      <c r="B10" t="str">
-        <v>173</v>
-      </c>
-      <c r="C10" t="str">
-        <v>sniperkraken007@gmail.com</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Veg</v>
-      </c>
-      <c r="E10">
-        <v>967</v>
-      </c>
-      <c r="F10" t="str">
-        <v>78a002bd-67a3-40bd-a81d-2d5b77f1ea67</v>
-      </c>
-      <c r="G10" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix:updated the email ui
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,10 +424,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Shravan R</v>
+        <v>Sniper Kraken</v>
       </c>
       <c r="B2" t="str">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C2" t="str">
         <v>sniperkraken007@gmail.com</v>
@@ -436,10 +436,10 @@
         <v>Veg</v>
       </c>
       <c r="E2">
-        <v>620</v>
+        <v>967</v>
       </c>
       <c r="F2" t="str">
-        <v>db484a6e-f78d-4fed-abd4-82d76873e244</v>
+        <v>78a002bd-67a3-40bd-a81d-2d5b77f1ea67</v>
       </c>
       <c r="G2" t="str">
         <v>No</v>
@@ -447,22 +447,22 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>shravan</v>
+        <v>PRICE</v>
       </c>
       <c r="B3" t="str">
-        <v>175</v>
+        <v>1mj23cs175</v>
       </c>
       <c r="C3" t="str">
-        <v>sniperkraken007@gmail.com</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D3" t="str">
         <v>Veg</v>
       </c>
       <c r="E3">
-        <v>816</v>
+        <v>684</v>
       </c>
       <c r="F3" t="str">
-        <v>0d1498e1-aef8-4097-912a-d99cab0f3b85</v>
+        <v>d0cec2a0-5a19-4276-bc0c-3b84a89e2e25</v>
       </c>
       <c r="G3" t="str">
         <v>No</v>
@@ -470,10 +470,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Shravan R</v>
+        <v>PRICE</v>
       </c>
       <c r="B4" t="str">
-        <v>175</v>
+        <v>1mj23cs175</v>
       </c>
       <c r="C4" t="str">
         <v>shravanramakunja@gmail.com</v>
@@ -482,10 +482,10 @@
         <v>Veg</v>
       </c>
       <c r="E4">
-        <v>507</v>
+        <v>762</v>
       </c>
       <c r="F4" t="str">
-        <v>0649a2f2-a85c-48e4-a00d-9c899f1139df</v>
+        <v>dc3ef832-fa1e-4131-a4e2-cea0cf26d538</v>
       </c>
       <c r="G4" t="str">
         <v>No</v>
@@ -493,22 +493,22 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>shravan</v>
+        <v>Shravan</v>
       </c>
       <c r="B5" t="str">
         <v>175</v>
       </c>
       <c r="C5" t="str">
-        <v>sniperkraken007@gmail.com</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D5" t="str">
         <v>Veg</v>
       </c>
       <c r="E5">
-        <v>321</v>
+        <v>151</v>
       </c>
       <c r="F5" t="str">
-        <v>160fc85e-1772-4f83-a920-0df6c85d5793</v>
+        <v>7287d48e-18ee-42a4-beea-af6d763bdbf9</v>
       </c>
       <c r="G5" t="str">
         <v>No</v>
@@ -519,73 +519,27 @@
         <v>Shravan R</v>
       </c>
       <c r="B6" t="str">
-        <v>175</v>
+        <v>1mj23cs175</v>
       </c>
       <c r="C6" t="str">
-        <v>sniperkraken007@gmail.com</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D6" t="str">
         <v>Veg</v>
       </c>
       <c r="E6">
-        <v>693</v>
+        <v>462</v>
       </c>
       <c r="F6" t="str">
-        <v>856d90b7-4506-4351-a017-2a16beaa2279</v>
+        <v>52a9b3ea-c70b-41b0-b883-f16301ccb27a</v>
       </c>
       <c r="G6" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Shravan R</v>
-      </c>
-      <c r="B7" t="str">
-        <v>175</v>
-      </c>
-      <c r="C7" t="str">
-        <v>shravanramakunja@gmail.com</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Non-Veg</v>
-      </c>
-      <c r="E7">
-        <v>746</v>
-      </c>
-      <c r="F7" t="str">
-        <v>eb258263-2334-4d6b-8b18-5bda969e00cd</v>
-      </c>
-      <c r="G7" t="str">
-        <v>No</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Sniper Kraken</v>
-      </c>
-      <c r="B8" t="str">
-        <v>173</v>
-      </c>
-      <c r="C8" t="str">
-        <v>sniperkraken007@gmail.com</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Veg</v>
-      </c>
-      <c r="E8">
-        <v>967</v>
-      </c>
-      <c r="F8" t="str">
-        <v>78a002bd-67a3-40bd-a81d-2d5b77f1ea67</v>
-      </c>
-      <c r="G8" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: 1.added the buttons  of dep,parents 2.added the maths algorithm to generate the seat number
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,67 +410,85 @@
         <v>Email</v>
       </c>
       <c r="D1" t="str">
-        <v>Food</v>
+        <v>Department</v>
       </c>
       <c r="E1" t="str">
         <v>Seat</v>
       </c>
       <c r="F1" t="str">
+        <v>Parents</v>
+      </c>
+      <c r="G1" t="str">
         <v>UniqueID</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>CheckedIn</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Food</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Sniper Kraken</v>
+        <v>PRICE</v>
       </c>
       <c r="B2" t="str">
-        <v>173</v>
+        <v>1mj23cs175</v>
       </c>
       <c r="C2" t="str">
-        <v>sniperkraken007@gmail.com</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2">
+        <v>684</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>d0cec2a0-5a19-4276-bc0c-3b84a89e2e25</v>
+      </c>
+      <c r="H2" t="str">
+        <v>No</v>
+      </c>
+      <c r="I2" t="str">
         <v>Veg</v>
-      </c>
-      <c r="E2">
-        <v>967</v>
-      </c>
-      <c r="F2" t="str">
-        <v>78a002bd-67a3-40bd-a81d-2d5b77f1ea67</v>
-      </c>
-      <c r="G2" t="str">
-        <v>No</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>PRICE</v>
+        <v>Shravan</v>
       </c>
       <c r="B3" t="str">
-        <v>1mj23cs175</v>
+        <v>175</v>
       </c>
       <c r="C3" t="str">
         <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3">
+        <v>151</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>7287d48e-18ee-42a4-beea-af6d763bdbf9</v>
+      </c>
+      <c r="H3" t="str">
+        <v>No</v>
+      </c>
+      <c r="I3" t="str">
         <v>Veg</v>
-      </c>
-      <c r="E3">
-        <v>684</v>
-      </c>
-      <c r="F3" t="str">
-        <v>d0cec2a0-5a19-4276-bc0c-3b84a89e2e25</v>
-      </c>
-      <c r="G3" t="str">
-        <v>No</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>PRICE</v>
+        <v>Shravan R</v>
       </c>
       <c r="B4" t="str">
         <v>1mj23cs175</v>
@@ -479,39 +497,51 @@
         <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D4" t="str">
-        <v>Veg</v>
-      </c>
-      <c r="E4">
-        <v>762</v>
+        <v>Computer Science and Design (CG)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>D022</v>
       </c>
       <c r="F4" t="str">
-        <v>dc3ef832-fa1e-4131-a4e2-cea0cf26d538</v>
+        <v>2</v>
       </c>
       <c r="G4" t="str">
+        <v>1f4d5944-a69e-4f85-8b55-782467c82b93</v>
+      </c>
+      <c r="H4" t="str">
         <v>No</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Shravan</v>
+        <v>Shravan R</v>
       </c>
       <c r="B5" t="str">
-        <v>175</v>
+        <v>1mj23cs175</v>
       </c>
       <c r="C5" t="str">
         <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D5" t="str">
-        <v>Veg</v>
-      </c>
-      <c r="E5">
-        <v>151</v>
+        <v>Computer Science and Design (CG)</v>
+      </c>
+      <c r="E5" t="str">
+        <v>D017</v>
       </c>
       <c r="F5" t="str">
-        <v>7287d48e-18ee-42a4-beea-af6d763bdbf9</v>
+        <v>2</v>
       </c>
       <c r="G5" t="str">
+        <v>1ada7c50-4b7f-4080-9edf-826e1780c684</v>
+      </c>
+      <c r="H5" t="str">
         <v>No</v>
+      </c>
+      <c r="I5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -525,21 +555,53 @@
         <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D6" t="str">
-        <v>Veg</v>
-      </c>
-      <c r="E6">
-        <v>462</v>
+        <v>Artificial Intelligence and Machine Learning (AI &amp; ML)</v>
+      </c>
+      <c r="E6" t="str">
+        <v>D079</v>
       </c>
       <c r="F6" t="str">
-        <v>52a9b3ea-c70b-41b0-b883-f16301ccb27a</v>
+        <v>2</v>
       </c>
       <c r="G6" t="str">
+        <v>fa05e5cc-e844-496d-a980-26cd2ba987c5</v>
+      </c>
+      <c r="H6" t="str">
+        <v>No</v>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Shravan R</v>
+      </c>
+      <c r="B7" t="str">
+        <v>1mj23cs175</v>
+      </c>
+      <c r="C7" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Aeronautical Engineering (AE)</v>
+      </c>
+      <c r="E7" t="str">
+        <v>A024</v>
+      </c>
+      <c r="F7" t="str">
+        <v>1</v>
+      </c>
+      <c r="G7" t="str">
+        <v>df1c576a-26b3-40a6-abd7-840600d947d9</v>
+      </c>
+      <c r="H7" t="str">
         <v>No</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: added new manual checkin
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -425,9 +425,35 @@
         <v>CheckedIn</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v xml:space="preserve">Shravan </v>
+      </c>
+      <c r="B2" t="str">
+        <v>1mj23cs175</v>
+      </c>
+      <c r="C2" t="str">
+        <v>shravanramakunja1@gmail.com</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Computer Science and Design (CG)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>D029</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2</v>
+      </c>
+      <c r="G2" t="str">
+        <v>467bcac6-69e7-4cbc-b34d-2d95c6f3b129</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: added the front end code
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -451,9 +451,87 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Shravan R</v>
+      </c>
+      <c r="B3" t="str">
+        <v>1mj23cs177</v>
+      </c>
+      <c r="C3" t="str">
+        <v>sniperkraken007@gmail.com</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Computer Science and Engineering and Data Science (CD)</v>
+      </c>
+      <c r="E3" t="str">
+        <v>D171</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2</v>
+      </c>
+      <c r="G3" t="str">
+        <v>a2bcb242-12ba-40c9-9020-9a466384e021</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Shravan R</v>
+      </c>
+      <c r="B4" t="str">
+        <v>1mj23cs177</v>
+      </c>
+      <c r="C4" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Computer Science and Design (CG)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>D170</v>
+      </c>
+      <c r="F4" t="str">
+        <v>1</v>
+      </c>
+      <c r="G4" t="str">
+        <v>b0a6d1f2-92d9-4d63-b5b3-8607ce07dcb6</v>
+      </c>
+      <c r="H4" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Shravan R</v>
+      </c>
+      <c r="B5" t="str">
+        <v>1mj23cs177</v>
+      </c>
+      <c r="C5" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Computer Science and Design (CG)</v>
+      </c>
+      <c r="E5" t="str">
+        <v>D151</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1</v>
+      </c>
+      <c r="G5" t="str">
+        <v>6fc1f5fd-095a-401c-8402-8a448af91db8</v>
+      </c>
+      <c r="H5" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat : added the removal of  duplication of error
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -419,7 +419,7 @@
         <v>Parents</v>
       </c>
       <c r="G1" t="str">
-        <v>UniqueID</v>
+        <v>uniqueId</v>
       </c>
       <c r="H1" t="str">
         <v>CheckedIn</v>
@@ -427,25 +427,25 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v xml:space="preserve">Shravan </v>
+        <v>Shravan R</v>
       </c>
       <c r="B2" t="str">
-        <v>1mj23cs175</v>
+        <v>1mj23cs177</v>
       </c>
       <c r="C2" t="str">
-        <v>shravanramakunja1@gmail.com</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D2" t="str">
-        <v>Computer Science and Design (CG)</v>
+        <v>Industrial IOT (IIoT)</v>
       </c>
       <c r="E2" t="str">
-        <v>D029</v>
+        <v>C014</v>
       </c>
       <c r="F2" t="str">
         <v>2</v>
       </c>
       <c r="G2" t="str">
-        <v>467bcac6-69e7-4cbc-b34d-2d95c6f3b129</v>
+        <v>ded408a8-b1ca-4a00-acc0-e38815883b3b</v>
       </c>
       <c r="H2" t="str">
         <v>Yes</v>
@@ -459,79 +459,183 @@
         <v>1mj23cs177</v>
       </c>
       <c r="C3" t="str">
-        <v>sniperkraken007@gmail.com</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D3" t="str">
-        <v>Computer Science and Engineering and Data Science (CD)</v>
+        <v>Industrial IOT (IIoT)</v>
       </c>
       <c r="E3" t="str">
-        <v>D171</v>
+        <v>C049</v>
       </c>
       <c r="F3" t="str">
         <v>2</v>
       </c>
       <c r="G3" t="str">
-        <v>a2bcb242-12ba-40c9-9020-9a466384e021</v>
+        <v>9bbdb4a1-1a34-4a1d-8818-328eb906f68a</v>
       </c>
       <c r="H3" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Shravan R</v>
+        <v>price</v>
       </c>
       <c r="B4" t="str">
-        <v>1mj23cs177</v>
+        <v>1mj23cs178</v>
       </c>
       <c r="C4" t="str">
         <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D4" t="str">
-        <v>Computer Science and Design (CG)</v>
+        <v>Chemical Engineering (CHE)</v>
       </c>
       <c r="E4" t="str">
-        <v>D170</v>
+        <v>B048</v>
       </c>
       <c r="F4" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" t="str">
-        <v>b0a6d1f2-92d9-4d63-b5b3-8607ce07dcb6</v>
+        <v>1831e4dc-07b6-413c-8497-7c3f934b5a29</v>
       </c>
       <c r="H4" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Shravan R</v>
+        <v>price</v>
       </c>
       <c r="B5" t="str">
-        <v>1mj23cs177</v>
+        <v>1mj23cs178</v>
       </c>
       <c r="C5" t="str">
         <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D5" t="str">
-        <v>Computer Science and Design (CG)</v>
+        <v>Chemical Engineering (CHE)</v>
       </c>
       <c r="E5" t="str">
-        <v>D151</v>
+        <v>B068</v>
       </c>
       <c r="F5" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="str">
-        <v>6fc1f5fd-095a-401c-8402-8a448af91db8</v>
+        <v>0694738f-c9b3-4d42-92c4-749ce193b950</v>
       </c>
       <c r="H5" t="str">
         <v>No</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v xml:space="preserve">Shravan </v>
+      </c>
+      <c r="B6" t="str">
+        <v>1mj23cs180</v>
+      </c>
+      <c r="C6" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Mechanical Engineering (ME)</v>
+      </c>
+      <c r="E6" t="str">
+        <v>A031</v>
+      </c>
+      <c r="F6" t="str">
+        <v>1</v>
+      </c>
+      <c r="G6" t="str">
+        <v>7c56d050-e1af-4319-8ce3-66ac6bd10600</v>
+      </c>
+      <c r="H6" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v xml:space="preserve">Shravan </v>
+      </c>
+      <c r="B7" t="str">
+        <v>1mj23cs180</v>
+      </c>
+      <c r="C7" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Mechanical Engineering (ME)</v>
+      </c>
+      <c r="E7" t="str">
+        <v>A009</v>
+      </c>
+      <c r="F7" t="str">
+        <v>1</v>
+      </c>
+      <c r="G7" t="str">
+        <v>3265bc86-ac34-4b20-8349-e05550fe78c5</v>
+      </c>
+      <c r="H7" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v xml:space="preserve">Shravan </v>
+      </c>
+      <c r="B8" t="str">
+        <v>1mj23cs180</v>
+      </c>
+      <c r="C8" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Mechanical Engineering (ME)</v>
+      </c>
+      <c r="E8" t="str">
+        <v>A001</v>
+      </c>
+      <c r="F8" t="str">
+        <v>1</v>
+      </c>
+      <c r="G8" t="str">
+        <v>06d77438-c8dd-49c2-b3af-1ced2adaadeb</v>
+      </c>
+      <c r="H8" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Shravan</v>
+      </c>
+      <c r="B9" t="str">
+        <v>1mj23cs177</v>
+      </c>
+      <c r="C9" t="str">
+        <v>shravanramakunja@okicici</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Information Science and Engineering (ISE)</v>
+      </c>
+      <c r="E9" t="str">
+        <v>E004</v>
+      </c>
+      <c r="F9" t="str">
+        <v>0</v>
+      </c>
+      <c r="G9" t="str">
+        <v>cf190324-1583-4852-816d-1f41398185ff</v>
+      </c>
+      <c r="H9" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat : added the filter in the admin dashboard
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -583,54 +583,54 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v xml:space="preserve">Shravan </v>
+        <v>Shravan R</v>
       </c>
       <c r="B8" t="str">
-        <v>1mj23cs180</v>
+        <v>1mj23cs175</v>
       </c>
       <c r="C8" t="str">
         <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D8" t="str">
-        <v>Mechanical Engineering (ME)</v>
+        <v>Electronics and Communication Engineering (ECE)</v>
       </c>
       <c r="E8" t="str">
-        <v>A001</v>
+        <v>C027</v>
       </c>
       <c r="F8" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" t="str">
-        <v>06d77438-c8dd-49c2-b3af-1ced2adaadeb</v>
+        <v>f132ee22-7d83-4130-9fd6-499e0f23e02a</v>
       </c>
       <c r="H8" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Shravan</v>
+        <v>Sniper Kraken</v>
       </c>
       <c r="B9" t="str">
-        <v>1mj23cs177</v>
+        <v>173</v>
       </c>
       <c r="C9" t="str">
-        <v>shravanramakunja@okicici</v>
+        <v>shravanramakunja@gmail.com</v>
       </c>
       <c r="D9" t="str">
-        <v>Information Science and Engineering (ISE)</v>
+        <v>Computer Science and Engineering (CSE)</v>
       </c>
       <c r="E9" t="str">
-        <v>E004</v>
+        <v>E019</v>
       </c>
       <c r="F9" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="str">
-        <v>cf190324-1583-4852-816d-1f41398185ff</v>
+        <v>2c17eccc-6080-4a00-a59e-fffc55fb182c</v>
       </c>
       <c r="H9" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix:changed the port of mail
</commit_message>
<xml_diff>
--- a/data/registrations.xlsx
+++ b/data/registrations.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -685,9 +685,87 @@
         <v>No</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>shravan</v>
+      </c>
+      <c r="B12" t="str">
+        <v>1mj23cs175</v>
+      </c>
+      <c r="C12" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Computer Science and Engineering and Data Science (CD)</v>
+      </c>
+      <c r="E12" t="str">
+        <v>D094</v>
+      </c>
+      <c r="F12" t="str">
+        <v>2</v>
+      </c>
+      <c r="G12" t="str">
+        <v>0286a371-208f-4596-809f-15fdda9922d8</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Shravan</v>
+      </c>
+      <c r="B13" t="str">
+        <v>1mj23cs175</v>
+      </c>
+      <c r="C13" t="str">
+        <v>shravanramakunja@gmail.com</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Mechanical Engineering (ME)</v>
+      </c>
+      <c r="E13" t="str">
+        <v>A023</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2</v>
+      </c>
+      <c r="G13" t="str">
+        <v>a99d7821-4389-47aa-8313-fb033fa6c6cf</v>
+      </c>
+      <c r="H13" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Shravan</v>
+      </c>
+      <c r="B14" t="str">
+        <v>1mj23cs177</v>
+      </c>
+      <c r="C14" t="str">
+        <v>sniperkraken007@gmail.com</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Information Science and Engineering (ISE)</v>
+      </c>
+      <c r="E14" t="str">
+        <v>E046</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2</v>
+      </c>
+      <c r="G14" t="str">
+        <v>dfd3c976-1d72-4f57-a378-4585dba775ae</v>
+      </c>
+      <c r="H14" t="str">
+        <v>No</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>